<commit_message>
feat(siswa): update Excel import template and validate rows with schema
Regenerates the student import template with all 36 saveSiswaSchema fields
</commit_message>
<xml_diff>
--- a/public/templates/template-import-siswa.xlsx
+++ b/public/templates/template-import-siswa.xlsx
@@ -397,58 +397,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:AJ3"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="23.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="17.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="25.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="25.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
+    <col min="22" max="22" width="17.83203125" customWidth="1"/>
+    <col min="23" max="23" width="21.83203125" customWidth="1"/>
+    <col min="24" max="24" width="18.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
+    <col min="26" max="26" width="20.83203125" customWidth="1"/>
+    <col min="27" max="27" width="25.83203125" customWidth="1"/>
+    <col min="28" max="28" width="30.83203125" customWidth="1"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1"/>
+    <col min="30" max="30" width="18.83203125" customWidth="1"/>
+    <col min="31" max="31" width="16.83203125" customWidth="1"/>
+    <col min="32" max="32" width="21.83203125" customWidth="1"/>
+    <col min="33" max="33" width="18.83203125" customWidth="1"/>
+    <col min="34" max="34" width="18.83203125" customWidth="1"/>
+    <col min="35" max="35" width="20.83203125" customWidth="1"/>
+    <col min="36" max="36" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Nama Lengkap*</v>
+        <v>nama_lengkap*</v>
       </c>
       <c r="B1" t="str">
-        <v>NIS*</v>
+        <v>nis</v>
       </c>
       <c r="C1" t="str">
-        <v>NISN*</v>
+        <v>nisn</v>
       </c>
       <c r="D1" t="str">
-        <v>Jenis Kelamin (L/P)</v>
+        <v>nama_panggilan</v>
       </c>
       <c r="E1" t="str">
-        <v>Tempat Lahir</v>
+        <v>jenis_kelamin</v>
       </c>
       <c r="F1" t="str">
-        <v>Tanggal Lahir (YYYY-MM-DD)</v>
+        <v>tempat_lahir</v>
       </c>
       <c r="G1" t="str">
-        <v>Nama Ayah</v>
+        <v>tanggal_lahir</v>
       </c>
       <c r="H1" t="str">
-        <v>Nama Ibu</v>
+        <v>agama</v>
       </c>
       <c r="I1" t="str">
-        <v>Nama Wali</v>
+        <v>status_dalam_keluarga</v>
       </c>
       <c r="J1" t="str">
-        <v>Telepon Wali</v>
+        <v>anak_ke</v>
       </c>
       <c r="K1" t="str">
-        <v>Alamat</v>
+        <v>alamat</v>
       </c>
       <c r="L1" t="str">
-        <v>Status (aktif/lulus/pindah/keluar)</v>
+        <v>alamat_dusun</v>
+      </c>
+      <c r="M1" t="str">
+        <v>alamat_rt</v>
+      </c>
+      <c r="N1" t="str">
+        <v>alamat_rw</v>
+      </c>
+      <c r="O1" t="str">
+        <v>alamat_desa</v>
+      </c>
+      <c r="P1" t="str">
+        <v>alamat_kecamatan</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>alamat_kabupaten_kota</v>
+      </c>
+      <c r="R1" t="str">
+        <v>nama_ayah</v>
+      </c>
+      <c r="S1" t="str">
+        <v>pekerjaan_ayah</v>
+      </c>
+      <c r="T1" t="str">
+        <v>nama_ibu</v>
+      </c>
+      <c r="U1" t="str">
+        <v>pekerjaan_ibu</v>
+      </c>
+      <c r="V1" t="str">
+        <v>no_telp_rumah</v>
+      </c>
+      <c r="W1" t="str">
+        <v>alamat_ortu_dusun</v>
+      </c>
+      <c r="X1" t="str">
+        <v>alamat_ortu_rt</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>alamat_ortu_rw</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>alamat_ortu_desa</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>alamat_ortu_kecamatan</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>alamat_ortu_kabupaten_kota</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>nama_wali</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>pekerjaan_wali</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>no_telp_wali</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>alamat_wali_dusun</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>alamat_wali_rt</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>alamat_wali_rw</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>alamat_wali_desa</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>status</v>
       </c>
     </row>
     <row r="2">
@@ -462,36 +558,218 @@
         <v>0051234567</v>
       </c>
       <c r="D2" t="str">
+        <v>Budi</v>
+      </c>
+      <c r="E2" t="str">
         <v>L</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Bandung</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>2008-05-12</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
+        <v>Islam</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Anak Tunggal</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Jl. Merdeka No. 10</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Dusun Suka Maju</v>
+      </c>
+      <c r="M2" t="str">
+        <v>001</v>
+      </c>
+      <c r="N2" t="str">
+        <v>002</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Desa Sukamaju</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Cibeunying</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Bandung</v>
+      </c>
+      <c r="R2" t="str">
         <v>Ahmad Santoso</v>
       </c>
-      <c r="H2" t="str">
+      <c r="S2" t="str">
+        <v>Wiraswasta</v>
+      </c>
+      <c r="T2" t="str">
         <v>Siti Aminah</v>
       </c>
-      <c r="I2" t="str">
-        <v>Ahmad Santoso</v>
-      </c>
-      <c r="J2" t="str">
+      <c r="U2" t="str">
+        <v>Ibu Rumah Tangga</v>
+      </c>
+      <c r="V2" t="str">
+        <v>022-1234567</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Dusun Suka Maju</v>
+      </c>
+      <c r="X2" t="str">
+        <v>001</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>002</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Desa Sukamaju</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Cibeunying</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Bandung</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>-</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>-</v>
+      </c>
+      <c r="AE2" t="str">
         <v>081234567890</v>
       </c>
-      <c r="K2" t="str">
-        <v>Jl. Merdeka No. 10, Bandung</v>
-      </c>
-      <c r="L2" t="str">
+      <c r="AF2" t="str">
+        <v>-</v>
+      </c>
+      <c r="AG2" t="str">
+        <v>-</v>
+      </c>
+      <c r="AH2" t="str">
+        <v>-</v>
+      </c>
+      <c r="AI2" t="str">
+        <v>-</v>
+      </c>
+      <c r="AJ2" t="str">
         <v>aktif</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Wajib, min 2 karakter</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Wajib isi NIS atau NISN</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Wajib isi NIS atau NISN</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>L atau P</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>Format YYYY-MM-DD</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Nama agama, mis. Islam</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v>Angka positif</v>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AG3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AH3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AI3" t="str">
+        <v>Opsional</v>
+      </c>
+      <c r="AJ3" t="str">
+        <v>aktif / lulus / pindah / keluar</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AJ3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>